<commit_message>
Migración Qt/PySide6, motor C++ Clipper2 y mejoras de nesting vs app original.
Incluye UI nativa (interface/qt), puente algorithm_bridge, fixes RTZ/transferencias, costos_prorrateo para placas sobrante, ajustes visuales, parsing geométrico y scanner.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/modules/Plates.xlsx
+++ b/modules/Plates.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,7 +493,7 @@
         <v>2047.69</v>
       </c>
       <c r="H2" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         <v>3917.16</v>
       </c>
       <c r="H8" t="n">
-        <v>1.64</v>
+        <v>1.65</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
         <v>4356.18</v>
       </c>
       <c r="H9" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1044,7 +1044,7 @@
         <v>1711.92</v>
       </c>
       <c r="H17" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1340,7 +1340,7 @@
         <v>1583.27</v>
       </c>
       <c r="H25" t="n">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1562,7 +1562,7 @@
         <v>23312.93</v>
       </c>
       <c r="H31" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -1636,7 +1636,7 @@
         <v>36173.36</v>
       </c>
       <c r="H33" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -2117,7 +2117,7 @@
         <v>14288.58</v>
       </c>
       <c r="H46" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -2376,7 +2376,7 @@
         <v>9066.549999999999</v>
       </c>
       <c r="H53" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -2413,7 +2413,7 @@
         <v>13599.84</v>
       </c>
       <c r="H54" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
         <v>30221.86</v>
       </c>
       <c r="H64" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
@@ -2894,7 +2894,7 @@
         <v>23964.08</v>
       </c>
       <c r="H67" t="n">
-        <v>2.24</v>
+        <v>2.25</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
@@ -3042,7 +3042,7 @@
         <v>14293.44</v>
       </c>
       <c r="H71" t="n">
-        <v>1.57</v>
+        <v>1.58</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
@@ -3116,7 +3116,7 @@
         <v>35388.1</v>
       </c>
       <c r="H73" t="n">
-        <v>1.62</v>
+        <v>1.63</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
@@ -3153,7 +3153,7 @@
         <v>72309.24000000001</v>
       </c>
       <c r="H74" t="n">
-        <v>2.21</v>
+        <v>2.22</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
@@ -3227,7 +3227,7 @@
         <v>13902.44</v>
       </c>
       <c r="H76" t="n">
-        <v>1.53</v>
+        <v>1.54</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
@@ -3556,7 +3556,7 @@
         <v>14293.44</v>
       </c>
       <c r="H85" t="n">
-        <v>1.57</v>
+        <v>1.58</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
@@ -3628,7 +3628,7 @@
         <v>28005.44</v>
       </c>
       <c r="H87" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
@@ -3665,9 +3665,46 @@
         <v>43596.5</v>
       </c>
       <c r="H88" t="n">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="I88" t="inlineStr">
+        <is>
+          <t>DISPONIBLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>SSTL 304</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>PLS042</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>120</v>
+      </c>
+      <c r="E89" t="n">
+        <v>48</v>
+      </c>
+      <c r="F89" t="n">
+        <v>1664.64</v>
+      </c>
+      <c r="G89" t="n">
+        <v>100</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0.003454</v>
+      </c>
+      <c r="I89" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>

</xml_diff>

<commit_message>
Corregir placas con mismo stock y consolidar mejoras del motor C++ de nesting.
Separa P1/P2 por identidad de hoja en el visor, añade sheet_integrity para deduplicar fantasmas, kerf 0.3 por defecto, overlays RTZ, export DXF/PDF y elimina el backend Cython legacy.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/modules/Plates.xlsx
+++ b/modules/Plates.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -567,7 +567,7 @@
         <v>1108.65</v>
       </c>
       <c r="H4" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
         <v>886.91</v>
       </c>
       <c r="H6" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -676,11 +676,11 @@
         <v>5890.5</v>
       </c>
       <c r="H7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>NO DISPONIBLE</t>
+          <t>DISPONIBLE</t>
         </is>
       </c>
     </row>
@@ -713,11 +713,11 @@
         <v>3917.16</v>
       </c>
       <c r="H8" t="n">
-        <v>1.65</v>
+        <v>1.67</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>NO DISPONIBLE</t>
+          <t>DISPONIBLE</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
         <v>4356.18</v>
       </c>
       <c r="H9" t="n">
-        <v>1.72</v>
+        <v>1.74</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -787,11 +787,11 @@
         <v>4814.63</v>
       </c>
       <c r="H10" t="n">
-        <v>1.52</v>
+        <v>1.54</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>NO DISPONIBLE</t>
+          <t>DISPONIBLE</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
         <v>6018.7</v>
       </c>
       <c r="H11" t="n">
-        <v>1.52</v>
+        <v>1.54</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -861,11 +861,11 @@
         <v>3578.5</v>
       </c>
       <c r="H12" t="n">
-        <v>1.58</v>
+        <v>1.6</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>NO DISPONIBLE</t>
+          <t>DISPONIBLE</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
         <v>2100</v>
       </c>
       <c r="H13" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
         <v>2605.75</v>
       </c>
       <c r="H14" t="n">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1081,7 +1081,7 @@
         <v>2161.05</v>
       </c>
       <c r="H18" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1118,7 +1118,7 @@
         <v>913.05</v>
       </c>
       <c r="H19" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
         <v>1213.23</v>
       </c>
       <c r="H20" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         <v>1360.23</v>
       </c>
       <c r="H21" t="n">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1229,7 +1229,7 @@
         <v>1108.65</v>
       </c>
       <c r="H22" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1303,11 +1303,11 @@
         <v>2259.32</v>
       </c>
       <c r="H24" t="n">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>NO DISPONIBLE</t>
+          <t>DISPONIBLE</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
         <v>7423.68</v>
       </c>
       <c r="H26" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1414,7 +1414,7 @@
         <v>11397.96</v>
       </c>
       <c r="H27" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1525,7 +1525,7 @@
         <v>11810.4</v>
       </c>
       <c r="H30" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1599,7 +1599,7 @@
         <v>18850.07</v>
       </c>
       <c r="H32" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
         <v>3711.84</v>
       </c>
       <c r="H34" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -1747,11 +1747,11 @@
         <v>4721.42</v>
       </c>
       <c r="H36" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>NO DISPONIBLE</t>
+          <t>DISPONIBLE</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
         <v>9490.27</v>
       </c>
       <c r="H37" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -1821,7 +1821,7 @@
         <v>11810.4</v>
       </c>
       <c r="H38" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -1895,7 +1895,7 @@
         <v>2788.9</v>
       </c>
       <c r="H40" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v>2464.36</v>
       </c>
       <c r="H42" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
         <v>3871.18</v>
       </c>
       <c r="H44" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2080,7 +2080,7 @@
         <v>19935.26</v>
       </c>
       <c r="H45" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>NO DISPONIBLE</t>
+          <t>DISPONIBLE</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2191,7 @@
         <v>5577.79</v>
       </c>
       <c r="H48" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
         <v>11511.17</v>
       </c>
       <c r="H49" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -2265,7 +2265,7 @@
         <v>7122.72</v>
       </c>
       <c r="H50" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -2302,7 +2302,7 @@
         <v>10686.08</v>
       </c>
       <c r="H51" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -2339,7 +2339,7 @@
         <v>13933.44</v>
       </c>
       <c r="H52" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -2450,7 +2450,7 @@
         <v>17726.24</v>
       </c>
       <c r="H55" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -2524,7 +2524,7 @@
         <v>4634.78</v>
       </c>
       <c r="H57" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
@@ -2561,7 +2561,7 @@
         <v>9498.299999999999</v>
       </c>
       <c r="H58" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
         <v>5677.55</v>
       </c>
       <c r="H59" t="n">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
@@ -2635,7 +2635,7 @@
         <v>11872.87</v>
       </c>
       <c r="H60" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
@@ -2672,7 +2672,7 @@
         <v>14768.32</v>
       </c>
       <c r="H61" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
         <v>22445.38</v>
       </c>
       <c r="H62" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
@@ -2746,7 +2746,7 @@
         <v>11872.87</v>
       </c>
       <c r="H63" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
         <v>17761.71</v>
       </c>
       <c r="H65" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
@@ -2857,7 +2857,7 @@
         <v>70743</v>
       </c>
       <c r="H66" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
@@ -2894,7 +2894,7 @@
         <v>23964.08</v>
       </c>
       <c r="H67" t="n">
-        <v>2.25</v>
+        <v>2.27</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
@@ -2931,7 +2931,7 @@
         <v>11086.62</v>
       </c>
       <c r="H68" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
@@ -3005,11 +3005,11 @@
         <v>10659.95</v>
       </c>
       <c r="H70" t="n">
-        <v>1.47</v>
+        <v>1.49</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>NO DISPONIBLE</t>
+          <t>DISPONIBLE</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
         <v>14293.44</v>
       </c>
       <c r="H71" t="n">
-        <v>1.58</v>
+        <v>1.6</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
@@ -3079,7 +3079,7 @@
         <v>15660.45</v>
       </c>
       <c r="H72" t="n">
-        <v>1.44</v>
+        <v>1.46</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
@@ -3116,11 +3116,11 @@
         <v>35388.1</v>
       </c>
       <c r="H73" t="n">
-        <v>1.63</v>
+        <v>1.65</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>NO DISPONIBLE</t>
+          <t>DISPONIBLE</t>
         </is>
       </c>
     </row>
@@ -3153,7 +3153,7 @@
         <v>72309.24000000001</v>
       </c>
       <c r="H74" t="n">
-        <v>2.22</v>
+        <v>2.24</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
@@ -3190,7 +3190,7 @@
         <v>9801.58</v>
       </c>
       <c r="H75" t="n">
-        <v>1.44</v>
+        <v>1.46</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
@@ -3227,7 +3227,7 @@
         <v>13902.44</v>
       </c>
       <c r="H76" t="n">
-        <v>1.54</v>
+        <v>1.55</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
@@ -3301,7 +3301,7 @@
         <v>23943.41</v>
       </c>
       <c r="H78" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
         <v>2464.36</v>
       </c>
       <c r="H80" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
@@ -3410,7 +3410,7 @@
         <v>1108.65</v>
       </c>
       <c r="H81" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
@@ -3482,7 +3482,7 @@
         <v>10686.08</v>
       </c>
       <c r="H83" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
@@ -3519,7 +3519,7 @@
         <v>17726.24</v>
       </c>
       <c r="H84" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
@@ -3556,7 +3556,7 @@
         <v>14293.44</v>
       </c>
       <c r="H85" t="n">
-        <v>1.58</v>
+        <v>1.6</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
@@ -3702,9 +3702,194 @@
         <v>100</v>
       </c>
       <c r="H89" t="n">
-        <v>0.003454</v>
+        <v>0.00349</v>
       </c>
       <c r="I89" t="inlineStr">
+        <is>
+          <t>DISPONIBLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>SCO015</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>144</v>
+      </c>
+      <c r="E90" t="n">
+        <v>6</v>
+      </c>
+      <c r="F90" t="n">
+        <v>69.77</v>
+      </c>
+      <c r="G90" t="n">
+        <v>130</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>DISPONIBLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>SLC041</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>144</v>
+      </c>
+      <c r="E91" t="n">
+        <v>2</v>
+      </c>
+      <c r="F91" t="n">
+        <v>23.26</v>
+      </c>
+      <c r="G91" t="n">
+        <v>100</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>DISPONIBLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>SCO014</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>144</v>
+      </c>
+      <c r="E92" t="n">
+        <v>5</v>
+      </c>
+      <c r="F92" t="n">
+        <v>58.14</v>
+      </c>
+      <c r="G92" t="n">
+        <v>130</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>DISPONIBLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>SCO003</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>144</v>
+      </c>
+      <c r="E93" t="n">
+        <v>4</v>
+      </c>
+      <c r="F93" t="n">
+        <v>46.51</v>
+      </c>
+      <c r="G93" t="n">
+        <v>50</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>DISPONIBLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>SCO002</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>144</v>
+      </c>
+      <c r="E94" t="n">
+        <v>3</v>
+      </c>
+      <c r="F94" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="G94" t="n">
+        <v>70</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I94" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>

</xml_diff>

<commit_message>
Mejorar export DXF, cobre solo largos y validar piezas en nesting.
Exporta circulos/arcos nativos desde AutoDXF, enruta CU unicamente a barras 144x2-6, y bloquea resultados incompletos para evitar piezas perdidas en nesteo general y largos.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/modules/Plates.xlsx
+++ b/modules/Plates.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I94"/>
+  <dimension ref="A1:J94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,6 +463,11 @@
           <t>Stock</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>/LB</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -500,6 +505,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -537,6 +543,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -567,13 +574,14 @@
         <v>1108.65</v>
       </c>
       <c r="H4" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -609,6 +617,7 @@
           <t>NO EXISTENTE</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -639,13 +648,14 @@
         <v>886.91</v>
       </c>
       <c r="H6" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -676,13 +686,14 @@
         <v>5890.5</v>
       </c>
       <c r="H7" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -713,13 +724,14 @@
         <v>3917.16</v>
       </c>
       <c r="H8" t="n">
-        <v>1.67</v>
+        <v>1.65</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -750,13 +762,14 @@
         <v>4356.18</v>
       </c>
       <c r="H9" t="n">
-        <v>1.74</v>
+        <v>1.72</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -787,13 +800,14 @@
         <v>4814.63</v>
       </c>
       <c r="H10" t="n">
-        <v>1.54</v>
+        <v>1.52</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -824,13 +838,14 @@
         <v>6018.7</v>
       </c>
       <c r="H11" t="n">
-        <v>1.54</v>
+        <v>1.52</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -861,13 +876,14 @@
         <v>3578.5</v>
       </c>
       <c r="H12" t="n">
-        <v>1.6</v>
+        <v>1.58</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -898,13 +914,14 @@
         <v>2100</v>
       </c>
       <c r="H13" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -935,13 +952,14 @@
         <v>2605.75</v>
       </c>
       <c r="H14" t="n">
-        <v>0.52</v>
+        <v>0.51</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -977,6 +995,7 @@
           <t>NO EXISTENTE</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1014,6 +1033,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1051,6 +1071,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1081,13 +1102,14 @@
         <v>2161.05</v>
       </c>
       <c r="H18" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1118,13 +1140,14 @@
         <v>913.05</v>
       </c>
       <c r="H19" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1155,13 +1178,14 @@
         <v>1213.23</v>
       </c>
       <c r="H20" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1192,13 +1216,14 @@
         <v>1360.23</v>
       </c>
       <c r="H21" t="n">
-        <v>0.52</v>
+        <v>0.51</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1229,13 +1254,14 @@
         <v>1108.65</v>
       </c>
       <c r="H22" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1273,6 +1299,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1303,13 +1330,14 @@
         <v>2259.32</v>
       </c>
       <c r="H24" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1347,6 +1375,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1377,13 +1406,14 @@
         <v>7423.68</v>
       </c>
       <c r="H26" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1414,13 +1444,14 @@
         <v>11397.96</v>
       </c>
       <c r="H27" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1458,6 +1489,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1495,6 +1527,7 @@
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1525,13 +1558,14 @@
         <v>11810.4</v>
       </c>
       <c r="H30" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1569,6 +1603,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1599,13 +1634,14 @@
         <v>18850.07</v>
       </c>
       <c r="H32" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1643,6 +1679,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1673,13 +1710,14 @@
         <v>3711.84</v>
       </c>
       <c r="H34" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1717,6 +1755,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1747,13 +1786,14 @@
         <v>4721.42</v>
       </c>
       <c r="H36" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1784,13 +1824,14 @@
         <v>9490.27</v>
       </c>
       <c r="H37" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1821,13 +1862,14 @@
         <v>11810.4</v>
       </c>
       <c r="H38" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1865,6 +1907,7 @@
           <t>NO EXISTENTE</t>
         </is>
       </c>
+      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1895,13 +1938,14 @@
         <v>2788.9</v>
       </c>
       <c r="H40" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1939,6 +1983,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1976,6 +2021,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2013,6 +2059,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2043,13 +2090,14 @@
         <v>3871.18</v>
       </c>
       <c r="H44" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2087,6 +2135,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2124,6 +2173,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2161,6 +2211,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2191,13 +2242,14 @@
         <v>5577.79</v>
       </c>
       <c r="H48" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2228,13 +2280,14 @@
         <v>11511.17</v>
       </c>
       <c r="H49" t="n">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2265,13 +2318,14 @@
         <v>7122.72</v>
       </c>
       <c r="H50" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2302,13 +2356,14 @@
         <v>10686.08</v>
       </c>
       <c r="H51" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2339,13 +2394,14 @@
         <v>13933.44</v>
       </c>
       <c r="H52" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2383,6 +2439,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2420,6 +2477,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2450,13 +2508,14 @@
         <v>17726.24</v>
       </c>
       <c r="H55" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2494,6 +2553,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2524,13 +2584,14 @@
         <v>4634.78</v>
       </c>
       <c r="H57" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2561,13 +2622,14 @@
         <v>9498.299999999999</v>
       </c>
       <c r="H58" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2598,13 +2660,14 @@
         <v>5677.55</v>
       </c>
       <c r="H59" t="n">
-        <v>0.52</v>
+        <v>0.51</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2635,13 +2698,14 @@
         <v>11872.87</v>
       </c>
       <c r="H60" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2672,13 +2736,14 @@
         <v>14768.32</v>
       </c>
       <c r="H61" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2709,13 +2774,14 @@
         <v>22445.38</v>
       </c>
       <c r="H62" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2746,13 +2812,14 @@
         <v>11872.87</v>
       </c>
       <c r="H63" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2790,6 +2857,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2827,6 +2895,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2857,13 +2926,14 @@
         <v>70743</v>
       </c>
       <c r="H66" t="n">
-        <v>0.63</v>
+        <v>0.62</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2894,13 +2964,14 @@
         <v>23964.08</v>
       </c>
       <c r="H67" t="n">
-        <v>2.27</v>
+        <v>2.25</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2931,13 +3002,14 @@
         <v>11086.62</v>
       </c>
       <c r="H68" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2975,6 +3047,7 @@
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3005,13 +3078,14 @@
         <v>10659.95</v>
       </c>
       <c r="H70" t="n">
-        <v>1.49</v>
+        <v>1.47</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3042,13 +3116,14 @@
         <v>14293.44</v>
       </c>
       <c r="H71" t="n">
-        <v>1.6</v>
+        <v>1.58</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3079,13 +3154,14 @@
         <v>15660.45</v>
       </c>
       <c r="H72" t="n">
-        <v>1.46</v>
+        <v>1.44</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3116,13 +3192,14 @@
         <v>35388.1</v>
       </c>
       <c r="H73" t="n">
-        <v>1.65</v>
+        <v>1.63</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3153,13 +3230,14 @@
         <v>72309.24000000001</v>
       </c>
       <c r="H74" t="n">
-        <v>2.24</v>
+        <v>2.22</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3190,13 +3268,14 @@
         <v>9801.58</v>
       </c>
       <c r="H75" t="n">
-        <v>1.46</v>
+        <v>1.45</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3227,13 +3306,14 @@
         <v>13902.44</v>
       </c>
       <c r="H76" t="n">
-        <v>1.55</v>
+        <v>1.54</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3271,6 +3351,7 @@
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3301,13 +3382,14 @@
         <v>23943.41</v>
       </c>
       <c r="H78" t="n">
-        <v>0.57</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3343,6 +3425,7 @@
           <t>NO EXISTENTE</t>
         </is>
       </c>
+      <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3380,6 +3463,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3410,13 +3494,14 @@
         <v>1108.65</v>
       </c>
       <c r="H81" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3452,6 +3537,7 @@
           <t>NO EXISTENTE</t>
         </is>
       </c>
+      <c r="J82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3482,13 +3568,14 @@
         <v>10686.08</v>
       </c>
       <c r="H83" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3519,13 +3606,14 @@
         <v>17726.24</v>
       </c>
       <c r="H84" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3556,13 +3644,14 @@
         <v>14293.44</v>
       </c>
       <c r="H85" t="n">
-        <v>1.6</v>
+        <v>1.58</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
           <t>NO DISPONIBLE</t>
         </is>
       </c>
+      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -3598,6 +3687,7 @@
           <t>NO EXISTENTE</t>
         </is>
       </c>
+      <c r="J86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3635,6 +3725,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3672,6 +3763,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3702,13 +3794,14 @@
         <v>100</v>
       </c>
       <c r="H89" t="n">
-        <v>0.00349</v>
+        <v>0.00346</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3746,6 +3839,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3783,6 +3877,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3820,6 +3915,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3857,6 +3953,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3894,6 +3991,7 @@
           <t>DISPONIBLE</t>
         </is>
       </c>
+      <c r="J94" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>